<commit_message>
Add new Jupyter notebook for local testing
</commit_message>
<xml_diff>
--- a/experiments/ThesisExperiment.xlsx
+++ b/experiments/ThesisExperiment.xlsx
@@ -14,7 +14,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <name val="Arial"/>
       <color rgb="FF000000"/>
@@ -40,6 +40,9 @@
       <color rgb="FF000000"/>
       <sz val="10"/>
     </font>
+    <font>
+      <b val="1"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -61,7 +64,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -77,6 +80,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -512,7 +516,7 @@
       <c r="AE1" s="3" t="n"/>
     </row>
     <row r="2">
-      <c r="A2" t="n">
+      <c r="A2" s="0" t="n">
         <v>1</v>
       </c>
       <c r="B2" s="4" t="inlineStr">
@@ -520,12 +524,12 @@
           <t>Naive RAG</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="0" t="inlineStr">
         <is>
           <t>Semantic Passage (200 tokens)</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D2" s="0" t="inlineStr">
         <is>
           <t>all-MiniLM-L6-v2</t>
         </is>
@@ -535,69 +539,69 @@
           <t>FAISS</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="F2" s="0" t="inlineStr">
         <is>
           <t>gpt-4o-mini</t>
         </is>
       </c>
-      <c r="G2" t="n">
+      <c r="G2" s="0" t="n">
         <v>0.7</v>
       </c>
-      <c r="H2" t="n">
+      <c r="H2" s="0" t="n">
         <v>0.5639999999999999</v>
       </c>
-      <c r="I2" t="n">
+      <c r="I2" s="0" t="n">
         <v>0.5639999999999999</v>
       </c>
-      <c r="J2" t="n">
+      <c r="J2" s="0" t="n">
         <v>0.5639999999999999</v>
       </c>
-      <c r="K2" t="n">
+      <c r="K2" s="0" t="n">
         <v>0.7</v>
       </c>
-      <c r="L2" t="n">
+      <c r="L2" s="0" t="n">
         <v>0.7</v>
       </c>
-      <c r="M2" t="n">
+      <c r="M2" s="0" t="n">
         <v>0.0463</v>
       </c>
-      <c r="N2" t="n">
+      <c r="N2" s="0" t="n">
         <v>0.0463</v>
       </c>
-      <c r="O2" t="n">
+      <c r="O2" s="0" t="n">
         <v>-0.2615</v>
       </c>
-      <c r="P2" t="n">
+      <c r="P2" s="0" t="n">
         <v>0.2242</v>
       </c>
-      <c r="Q2" t="n">
+      <c r="Q2" s="0" t="n">
         <v>-0.0305</v>
       </c>
-      <c r="R2" t="n">
+      <c r="R2" s="0" t="n">
         <v>0.6</v>
       </c>
-      <c r="S2" t="n">
+      <c r="S2" s="0" t="n">
         <v>0.6333</v>
       </c>
-      <c r="T2" t="n">
+      <c r="T2" s="0" t="n">
         <v>0.6333</v>
       </c>
-      <c r="U2" t="n">
+      <c r="U2" s="0" t="n">
         <v>0.4289</v>
       </c>
-      <c r="V2" t="n">
+      <c r="V2" s="0" t="n">
         <v>0.2874</v>
       </c>
-      <c r="W2" t="n">
+      <c r="W2" s="0" t="n">
         <v>0.6667</v>
       </c>
-      <c r="X2" t="n">
+      <c r="X2" s="0" t="n">
         <v>0.9399999999999999</v>
       </c>
-      <c r="Y2" t="n">
+      <c r="Y2" s="0" t="n">
         <v>0.4112</v>
       </c>
-      <c r="Z2" t="n">
+      <c r="Z2" s="0" t="n">
         <v>0.3267</v>
       </c>
     </row>
@@ -752,9 +756,382 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:Z20"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
-  <sheetData/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>SN</t>
+        </is>
+      </c>
+      <c r="B1" s="7" t="inlineStr">
+        <is>
+          <t>RAG Name</t>
+        </is>
+      </c>
+      <c r="C1" s="7" t="inlineStr">
+        <is>
+          <t>Chunking Technique</t>
+        </is>
+      </c>
+      <c r="D1" s="7" t="inlineStr">
+        <is>
+          <t>Embedding</t>
+        </is>
+      </c>
+      <c r="E1" s="7" t="inlineStr">
+        <is>
+          <t>VectorDB</t>
+        </is>
+      </c>
+      <c r="F1" s="7" t="inlineStr">
+        <is>
+          <t>Generator Model</t>
+        </is>
+      </c>
+      <c r="G1" s="7" t="inlineStr">
+        <is>
+          <t>Accuracy</t>
+        </is>
+      </c>
+      <c r="H1" s="7" t="inlineStr">
+        <is>
+          <t>Precision</t>
+        </is>
+      </c>
+      <c r="I1" s="7" t="inlineStr">
+        <is>
+          <t>Recall</t>
+        </is>
+      </c>
+      <c r="J1" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="K1" s="7" t="inlineStr">
+        <is>
+          <t>Token F1</t>
+        </is>
+      </c>
+      <c r="L1" s="7" t="inlineStr">
+        <is>
+          <t>Exact Match</t>
+        </is>
+      </c>
+      <c r="M1" s="7" t="inlineStr">
+        <is>
+          <t>ROUGE-1</t>
+        </is>
+      </c>
+      <c r="N1" s="7" t="inlineStr">
+        <is>
+          <t>ROUGE-L</t>
+        </is>
+      </c>
+      <c r="O1" s="7" t="inlineStr">
+        <is>
+          <t>BERTScore P</t>
+        </is>
+      </c>
+      <c r="P1" s="7" t="inlineStr">
+        <is>
+          <t>BERTScore R</t>
+        </is>
+      </c>
+      <c r="Q1" s="7" t="inlineStr">
+        <is>
+          <t>BERTScore F1</t>
+        </is>
+      </c>
+      <c r="R1" s="7" t="inlineStr">
+        <is>
+          <t>Recall@3</t>
+        </is>
+      </c>
+      <c r="S1" s="7" t="inlineStr">
+        <is>
+          <t>Recall@5</t>
+        </is>
+      </c>
+      <c r="T1" s="7" t="inlineStr">
+        <is>
+          <t>Recall@10</t>
+        </is>
+      </c>
+      <c r="U1" s="7" t="inlineStr">
+        <is>
+          <t>MRR</t>
+        </is>
+      </c>
+      <c r="V1" s="7" t="inlineStr">
+        <is>
+          <t>RAGAS Faithfulness</t>
+        </is>
+      </c>
+      <c r="W1" s="7" t="inlineStr">
+        <is>
+          <t>RAGAS Hallucination Rate</t>
+        </is>
+      </c>
+      <c r="X1" s="7" t="inlineStr">
+        <is>
+          <t>RAGAS Answer Relevance</t>
+        </is>
+      </c>
+      <c r="Y1" s="7" t="inlineStr">
+        <is>
+          <t>RAGAS Context Precision</t>
+        </is>
+      </c>
+      <c r="Z1" s="7" t="inlineStr">
+        <is>
+          <t>RAGAS Context Recall</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Naive RAG</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>FAISS</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Naive RAG</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>FAISS</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Naive RAG</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>FAISS</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Naive RAG</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>FAISS</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Sparse RAG</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>FAISS</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Sparse RAG</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>FAISS</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Sparse RAG</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>FAISS</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Sparse RAG</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>FAISS</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Hybrid RAG</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>FAISS</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Hybrid RAG</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>FAISS</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Hybrid RAG</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>FAISS</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Hybrid RAG</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>FAISS</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Multi-Hop RAG</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>FAISS</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Multi-Hop RAG</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>FAISS</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Multi-Hop RAG</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>FAISS</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Multi-Hop RAG</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>FAISS</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>